<commit_message>
Update model after TeSS dev call 2026-07-01
</commit_message>
<xml_diff>
--- a/models/minimum-metadata-model.xlsx
+++ b/models/minimum-metadata-model.xlsx
@@ -578,7 +578,7 @@
     <t>Timezone</t>
   </si>
   <si>
-    <t>RFC 822 4-digit time zone [TBC]</t>
+    <t>IANA RFC 6557</t>
   </si>
   <si>
     <t>EVENT PROPOSED: The timezone [select from list]</t>
@@ -1564,8 +1564,8 @@
         <v>58</v>
       </c>
       <c r="F10" s="13"/>
-      <c r="G10" s="9" t="s">
-        <v>16</v>
+      <c r="G10" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>62</v>
@@ -2096,8 +2096,8 @@
         <v>128</v>
       </c>
       <c r="F32" s="17"/>
-      <c r="G32" s="9" t="s">
-        <v>16</v>
+      <c r="G32" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="14" t="s">

</xml_diff>